<commit_message>
simplification de la fonction de prédiction electre_tri
</commit_message>
<xml_diff>
--- a/data/produits.xlsx
+++ b/data/produits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samy/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6A5AC81-13F4-664F-A58E-3AD16776E3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8977B7A-47E1-2E43-8F23-FFBF41E5D0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6060" yWindow="-20980" windowWidth="38400" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BD" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="255">
   <si>
     <t>Produit</t>
   </si>
@@ -554,6 +554,240 @@
   </si>
   <si>
     <t>452 mg</t>
+  </si>
+  <si>
+    <t>Grains d epautre complet bio – Bio sonne – 750 g</t>
+  </si>
+  <si>
+    <t>1443 kj / 345 kcal</t>
+  </si>
+  <si>
+    <t>Oui</t>
+  </si>
+  <si>
+    <t>Cannellones complètes – Naturaline – 250 g</t>
+  </si>
+  <si>
+    <t>374 kcal / 1 565 kJ</t>
+  </si>
+  <si>
+    <t>Semoule De Blé Fine Complète Bio – La Vie Claire – 500 g</t>
+  </si>
+  <si>
+    <t>347,6 kcal / 1 470,8 kJ</t>
+  </si>
+  <si>
+    <t>A+</t>
+  </si>
+  <si>
+    <t>Tartines Bio craquantes aux pois chiches sans gluten – Ekibio – 150 g, 2 sachets</t>
+  </si>
+  <si>
+    <t>378 kcal / 1 582 kJ</t>
+  </si>
+  <si>
+    <t>muesli ensoleillé fruit d'été – bjorg – 375 g</t>
+  </si>
+  <si>
+    <t>372 kcal / 1 567 kJ</t>
+  </si>
+  <si>
+    <t>Farine d'épeautre T80 – MelBio – 1 kg</t>
+  </si>
+  <si>
+    <t>348 kcal / 1 456 kJ</t>
+  </si>
+  <si>
+    <t>Pizza pâte complète</t>
+  </si>
+  <si>
+    <t>232 kcal / 971 kJ</t>
+  </si>
+  <si>
+    <t>Non</t>
+  </si>
+  <si>
+    <t>Epicerie / Epicerie Sucrée / Galettes Riz Et Céréales – Primeal – 100 g</t>
+  </si>
+  <si>
+    <t>372 kcal / 1 556 kJ</t>
+  </si>
+  <si>
+    <t>Kallo Natures Rice Cake imp – kallø – 130 g</t>
+  </si>
+  <si>
+    <t>394 kcal / 1 620 kJ</t>
+  </si>
+  <si>
+    <t>Crème sésame noir – Jean Hervé – 350 g</t>
+  </si>
+  <si>
+    <t>626 kcal / 2 587 kJ</t>
+  </si>
+  <si>
+    <t>Karéléa céréales figues – 150 g</t>
+  </si>
+  <si>
+    <t>433 kcal / 1819 kJ</t>
+  </si>
+  <si>
+    <t>Ravioli – Belle France – 400 g e</t>
+  </si>
+  <si>
+    <t>98 kcal / 410 kJ</t>
+  </si>
+  <si>
+    <t>Farine de millet brun – BIOSAGESSE – 500 g</t>
+  </si>
+  <si>
+    <t>377 kcal / 1595 kJ</t>
+  </si>
+  <si>
+    <t>Polenta de féverole complète – Graine de choc – 1 kg</t>
+  </si>
+  <si>
+    <t>319 kcal / 1345 kJ</t>
+  </si>
+  <si>
+    <t>Porridge figue framboise – Bjorg – 375 g</t>
+  </si>
+  <si>
+    <t>363 kcal / 1 528 kJ</t>
+  </si>
+  <si>
+    <t>Penne Rigate au blé complet bio – Casino – 500 g</t>
+  </si>
+  <si>
+    <t>346 kcal / 1 461 kJ</t>
+  </si>
+  <si>
+    <t>Granola amande &amp; miel – Aline &amp; Olivier – 310 g</t>
+  </si>
+  <si>
+    <t>447 kcal / 1870 kJ</t>
+  </si>
+  <si>
+    <t>Mix' Galettes petit épeautre &amp; soja – Priméal – 250 g</t>
+  </si>
+  <si>
+    <t>392 kcal / 1640 kJ</t>
+  </si>
+  <si>
+    <t>Céréales Muesli floconneux chocolat noir et graines de courge 375g – U – 375 g</t>
+  </si>
+  <si>
+    <t>388 kcal / 1 628 kJ</t>
+  </si>
+  <si>
+    <t>mélange pour pain aux graines – Adams Brot – 250 g</t>
+  </si>
+  <si>
+    <t>250 kcal / 1046.7 kJ</t>
+  </si>
+  <si>
+    <t>Galettes à base d'épeautre 130g – U – 130 g</t>
+  </si>
+  <si>
+    <t>362 kcal / 1531 kJ</t>
+  </si>
+  <si>
+    <t>Pain complet de seigle aux graines de tournesol – Céréal BIO – 500 g</t>
+  </si>
+  <si>
+    <t>214 kcal / 895 kJ</t>
+  </si>
+  <si>
+    <t>Chickpea - pasta organic – Kazidomi – 250 g</t>
+  </si>
+  <si>
+    <t>336 kcal / 1406 kJ</t>
+  </si>
+  <si>
+    <t>Wraps intégral Blé complet – Mission</t>
+  </si>
+  <si>
+    <t>290 kcal / 1226 kJ</t>
+  </si>
+  <si>
+    <t>Mélange de 5 céréales – Monoprix Bio – 500 g</t>
+  </si>
+  <si>
+    <t>350 kcal / 1480 kJ</t>
+  </si>
+  <si>
+    <t>4 Petits Pains sans Sel – Picard – 160 g</t>
+  </si>
+  <si>
+    <t>244 kcal / 1021 kJ</t>
+  </si>
+  <si>
+    <t>Polenta aux cepes – Moulin des Moines – 250 g</t>
+  </si>
+  <si>
+    <t>367 kcal / 1536 kJ</t>
+  </si>
+  <si>
+    <t>Grissino gusto classico – Vialatina – 200 g e</t>
+  </si>
+  <si>
+    <t>411 kcal / 1720 kJ</t>
+  </si>
+  <si>
+    <t>Couscous au chanvre – Priméal – 500 g</t>
+  </si>
+  <si>
+    <t>389 kcal / 1640 kJ</t>
+  </si>
+  <si>
+    <t>Trésor – Kellogg's – 410 g</t>
+  </si>
+  <si>
+    <t>433 kcal / 1812 kJ</t>
+  </si>
+  <si>
+    <t>Boules de céréales au chocolat – Eco+ – 750 g</t>
+  </si>
+  <si>
+    <t>372 kcal / 1556 kJ</t>
+  </si>
+  <si>
+    <t>Corn Flakes sucrées – Eco + – 750 g e (2 * 375 g)</t>
+  </si>
+  <si>
+    <t>387 kcal / 1619 kJ</t>
+  </si>
+  <si>
+    <t>Cereales – Nestlé</t>
+  </si>
+  <si>
+    <t>380 kcal / 1590 kJ</t>
+  </si>
+  <si>
+    <t>Céréales</t>
+  </si>
+  <si>
+    <t>318.8 kcal / 1334.0 kJ</t>
+  </si>
+  <si>
+    <t>Croc'Choco Blanc – Lucien Georgelin – 375g</t>
+  </si>
+  <si>
+    <t>435 kcal / 1820 kJ</t>
+  </si>
+  <si>
+    <t>Céréales Extra Kellogg's Pépites Chocolat au lait – 500 g</t>
+  </si>
+  <si>
+    <t>484 kcal / 2026 kJ</t>
+  </si>
+  <si>
+    <t>Céréales Extra Pepites Kellogg's Chocolat au lait – 800 g</t>
+  </si>
+  <si>
+    <t>Kelloggs extra aux 3 fruits rouges – Kellogg's – 500g</t>
+  </si>
+  <si>
+    <t>495 kcal / 2074 kJ</t>
   </si>
 </sst>
 </file>
@@ -582,12 +816,18 @@
       <name val="Calibri (Corps)"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -617,29 +857,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -945,10 +1184,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N64"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="45.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="69.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.83203125" bestFit="1" customWidth="1"/>
@@ -1008,1106 +1247,2789 @@
       </c>
     </row>
     <row r="2" spans="1:14" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="4">
         <v>7</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" s="4">
         <v>50</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="6">
         <v>0.16</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="4">
         <v>9</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="4">
         <v>57</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="4">
-        <v>0</v>
-      </c>
-      <c r="I4" s="3">
+      <c r="H4" s="6">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4">
         <v>7</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L4" s="3">
+      <c r="L4" s="4">
         <v>58</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H5" s="4">
-        <v>0</v>
-      </c>
-      <c r="I5" s="3">
+      <c r="H5" s="6">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4">
         <v>8</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="3">
+      <c r="L5" s="4">
         <v>45</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N5">
+      <c r="N5" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="3">
         <v>8.4399999999999996E-3</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="4">
         <v>10</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L6" s="3">
+      <c r="L6" s="4">
         <v>45</v>
       </c>
-      <c r="M6" t="s">
+      <c r="M6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N6">
+      <c r="N6" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="5">
-        <v>0</v>
-      </c>
-      <c r="I7" s="3">
+      <c r="H7" s="6">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4">
         <v>10</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L7" s="3">
+      <c r="L7" s="4">
         <v>45</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="6">
         <v>0.35</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="4">
         <v>4</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L8" s="3">
+      <c r="L8" s="4">
         <v>45</v>
       </c>
-      <c r="M8" t="s">
+      <c r="M8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N8">
+      <c r="N8" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="H9" s="4">
-        <v>0</v>
-      </c>
-      <c r="I9" s="3">
+      <c r="H9" s="6">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4">
         <v>6</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L9" s="3">
+      <c r="L9" s="4">
         <v>45</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N9">
+      <c r="N9" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="4">
-        <v>0</v>
-      </c>
-      <c r="I10" s="3">
+      <c r="H10" s="6">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4">
         <v>7</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L10" s="3">
+      <c r="L10" s="4">
         <v>45</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N10">
+      <c r="N10" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="H11" s="4">
-        <v>0</v>
-      </c>
-      <c r="I11" s="3">
+      <c r="H11" s="6">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4">
         <v>3</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L11" s="3">
+      <c r="L11" s="4">
         <v>45</v>
       </c>
-      <c r="M11" t="s">
+      <c r="M11" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N11">
+      <c r="N11" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="4">
-        <v>0</v>
-      </c>
-      <c r="I12" s="3">
+      <c r="H12" s="6">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4">
         <v>7</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K12" t="s">
+      <c r="K12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L12" s="3">
+      <c r="L12" s="4">
         <v>46</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M12" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N12">
+      <c r="N12" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="H13" s="4">
-        <v>0</v>
-      </c>
-      <c r="I13" s="3">
+      <c r="H13" s="6">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4">
         <v>8</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K13" t="s">
+      <c r="K13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L13" s="3">
+      <c r="L13" s="4">
         <v>45</v>
       </c>
-      <c r="M13" t="s">
+      <c r="M13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N13">
+      <c r="N13" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="H14" s="4">
-        <v>0</v>
-      </c>
-      <c r="I14" s="3">
+      <c r="H14" s="6">
+        <v>0</v>
+      </c>
+      <c r="I14" s="4">
         <v>8</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L14" s="3">
+      <c r="L14" s="4">
         <v>57</v>
       </c>
-      <c r="M14" t="s">
+      <c r="M14" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N14">
+      <c r="N14" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="H15" s="4">
+      <c r="H15" s="6">
         <v>0.18</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="4">
         <v>9</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K15" t="s">
+      <c r="K15" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L15" s="3">
+      <c r="L15" s="4">
         <v>57</v>
       </c>
-      <c r="M15" t="s">
+      <c r="M15" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N15">
+      <c r="N15" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="H16" s="4">
-        <v>0</v>
-      </c>
-      <c r="I16" s="3">
+      <c r="H16" s="6">
+        <v>0</v>
+      </c>
+      <c r="I16" s="4">
         <v>8</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K16" t="s">
+      <c r="K16" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L16" s="3">
+      <c r="L16" s="4">
         <v>50</v>
       </c>
-      <c r="M16" t="s">
+      <c r="M16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="N16">
+      <c r="N16" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="A17" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="H17" s="4">
-        <v>0</v>
-      </c>
-      <c r="I17" s="3">
+      <c r="H17" s="6">
+        <v>0</v>
+      </c>
+      <c r="I17" s="4">
         <v>9</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K17" t="s">
+      <c r="K17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="L17" s="3">
+      <c r="L17" s="4">
         <v>15</v>
       </c>
-      <c r="M17" t="s">
+      <c r="M17" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N17">
+      <c r="N17" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="H18" s="4">
-        <v>0</v>
-      </c>
-      <c r="I18" s="3">
+      <c r="H18" s="6">
+        <v>0</v>
+      </c>
+      <c r="I18" s="4">
         <v>6</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J18" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K18" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="L18" s="3">
+      <c r="L18" s="4">
         <v>30</v>
       </c>
-      <c r="M18" t="s">
+      <c r="M18" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N18">
+      <c r="N18" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="6">
         <v>0.18</v>
       </c>
-      <c r="I19" s="3">
+      <c r="I19" s="4">
         <v>9</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K19" t="s">
+      <c r="K19" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="L19" s="3">
+      <c r="L19" s="4">
         <v>62</v>
       </c>
-      <c r="M19" t="s">
+      <c r="M19" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N19">
+      <c r="N19" s="4">
         <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="H20" s="4">
-        <v>0</v>
-      </c>
-      <c r="I20" s="3">
+      <c r="H20" s="6">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4">
         <v>10</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K20" t="s">
+      <c r="K20" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="L20" s="3">
+      <c r="L20" s="4">
         <v>25</v>
       </c>
-      <c r="M20" t="s">
+      <c r="M20" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N20">
+      <c r="N20" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="A21" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="3">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="I21" s="3">
+      <c r="I21" s="4">
         <v>10</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K21" t="s">
-        <v>129</v>
-      </c>
-      <c r="L21" s="3">
+      <c r="K21" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="L21" s="4">
         <v>77</v>
       </c>
-      <c r="M21" t="s">
+      <c r="M21" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N21">
+      <c r="N21" s="4">
         <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="A22" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="H22" s="6">
+      <c r="H22" s="3">
         <v>8.6499999999999994E-2</v>
       </c>
-      <c r="I22" s="3">
+      <c r="I22" s="4">
         <v>19</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J22" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="K22" t="s">
+      <c r="K22" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="L22" s="3">
+      <c r="L22" s="4">
         <v>25</v>
       </c>
-      <c r="M22" t="s">
+      <c r="M22" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N22">
+      <c r="N22" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H23" s="4">
-        <v>0</v>
-      </c>
-      <c r="I23" s="3">
+      <c r="H23" s="6">
+        <v>0</v>
+      </c>
+      <c r="I23" s="4">
         <v>19</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="K23" t="s">
+      <c r="K23" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="L23" s="3">
+      <c r="L23" s="4">
         <v>25</v>
       </c>
-      <c r="M23" t="s">
+      <c r="M23" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N23">
+      <c r="N23" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="H24" s="4">
-        <v>0</v>
-      </c>
-      <c r="I24" s="3">
+      <c r="H24" s="6">
+        <v>0</v>
+      </c>
+      <c r="I24" s="4">
         <v>19</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="K24" t="s">
+      <c r="K24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="L24" s="3">
+      <c r="L24" s="4">
         <v>29</v>
       </c>
-      <c r="M24" t="s">
+      <c r="M24" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N24">
+      <c r="N24" s="4">
         <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="3">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="I25" s="3">
+      <c r="I25" s="4">
         <v>19</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="K25" t="s">
+      <c r="K25" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="L25" s="3">
+      <c r="L25" s="4">
         <v>25</v>
       </c>
-      <c r="M25" t="s">
+      <c r="M25" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N25">
+      <c r="N25" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="3">
         <v>2.5829999999999999E-2</v>
       </c>
-      <c r="I26" s="3">
+      <c r="I26" s="4">
         <v>19</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="K26" t="s">
+      <c r="K26" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="L26" s="3">
+      <c r="L26" s="4">
         <v>20</v>
       </c>
-      <c r="M26" t="s">
+      <c r="M26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="N26">
+      <c r="N26" s="4">
         <v>8</v>
       </c>
     </row>
-    <row r="64" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A27" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C27" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="D27" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="E27" s="8">
+        <v>0</v>
+      </c>
+      <c r="F27" s="8">
+        <v>17</v>
+      </c>
+      <c r="G27" s="8">
+        <v>10</v>
+      </c>
+      <c r="H27" s="8">
+        <v>0</v>
+      </c>
+      <c r="I27" s="8">
+        <v>-10</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L27" s="8">
+        <v>95</v>
+      </c>
+      <c r="M27" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N27" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A28" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="C28" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="D28" s="8">
+        <v>6.8</v>
+      </c>
+      <c r="E28" s="8">
+        <v>0.11</v>
+      </c>
+      <c r="F28" s="8">
+        <v>17.7</v>
+      </c>
+      <c r="G28" s="8">
+        <v>11.2</v>
+      </c>
+      <c r="H28" s="8">
+        <v>0</v>
+      </c>
+      <c r="I28" s="8">
+        <v>-7</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K28" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L28" s="8">
+        <v>82</v>
+      </c>
+      <c r="M28" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N28" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A29" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="C29" s="8">
+        <v>0.43</v>
+      </c>
+      <c r="D29" s="8">
+        <v>0.41</v>
+      </c>
+      <c r="E29" s="8">
+        <v>0</v>
+      </c>
+      <c r="F29" s="8">
+        <v>12.4</v>
+      </c>
+      <c r="G29" s="8">
+        <v>8</v>
+      </c>
+      <c r="H29" s="8">
+        <v>0</v>
+      </c>
+      <c r="I29" s="8">
+        <v>-9</v>
+      </c>
+      <c r="J29" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K29" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L29" s="8">
+        <v>86</v>
+      </c>
+      <c r="M29" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N29" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C30" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="D30" s="8">
+        <v>1.6</v>
+      </c>
+      <c r="E30" s="8">
+        <v>0.48</v>
+      </c>
+      <c r="F30" s="8">
+        <v>14.8</v>
+      </c>
+      <c r="G30" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8">
+        <v>-5</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K30" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L30" s="8">
+        <v>91</v>
+      </c>
+      <c r="M30" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N30" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A31" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="C31" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="D31" s="8">
+        <v>2.9</v>
+      </c>
+      <c r="E31" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="F31" s="8">
+        <v>13.1</v>
+      </c>
+      <c r="G31" s="8">
+        <v>10.8</v>
+      </c>
+      <c r="H31" s="8">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="I31" s="8">
+        <v>-6</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L31" s="8">
+        <v>82</v>
+      </c>
+      <c r="M31" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N31" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A32" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="C32" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="D32" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="E32" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="F32" s="8">
+        <v>13.4</v>
+      </c>
+      <c r="G32" s="8">
+        <v>7.2</v>
+      </c>
+      <c r="H32" s="8">
+        <v>0</v>
+      </c>
+      <c r="I32" s="8">
+        <v>-9</v>
+      </c>
+      <c r="J32" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L32" s="8">
+        <v>94</v>
+      </c>
+      <c r="M32" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N32" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A33" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="C33" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="D33" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="E33" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="F33" s="8">
+        <v>8</v>
+      </c>
+      <c r="G33" s="8">
+        <v>1.61</v>
+      </c>
+      <c r="H33" s="8">
+        <v>0</v>
+      </c>
+      <c r="I33" s="8">
+        <v>-1</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K33" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L33" s="8">
+        <v>91</v>
+      </c>
+      <c r="M33" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N33" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A34" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C34" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="D34" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="E34" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="F34" s="8">
+        <v>11.4</v>
+      </c>
+      <c r="G34" s="8">
+        <v>7.7</v>
+      </c>
+      <c r="H34" s="8">
+        <v>0</v>
+      </c>
+      <c r="I34" s="8">
+        <v>-3</v>
+      </c>
+      <c r="J34" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K34" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L34" s="8">
+        <v>87</v>
+      </c>
+      <c r="M34" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N34" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A35" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="C35" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="D35" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="E35" s="8">
+        <v>0</v>
+      </c>
+      <c r="F35" s="8">
+        <v>8.5</v>
+      </c>
+      <c r="G35" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="H35" s="8">
+        <v>0</v>
+      </c>
+      <c r="I35" s="8">
+        <v>0</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="L35" s="8">
+        <v>64</v>
+      </c>
+      <c r="M35" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N35" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A36" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="C36" s="8">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="D36" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="E36" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="F36" s="8">
+        <v>24.3</v>
+      </c>
+      <c r="G36" s="8">
+        <v>12.5</v>
+      </c>
+      <c r="H36" s="8">
+        <v>0</v>
+      </c>
+      <c r="I36" s="8">
+        <v>-8</v>
+      </c>
+      <c r="J36" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="L36" s="8">
+        <v>51</v>
+      </c>
+      <c r="M36" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N36" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A37" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="C37" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="D37" s="8">
+        <v>14</v>
+      </c>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8">
+        <v>7.7</v>
+      </c>
+      <c r="G37" s="8">
+        <v>7.8</v>
+      </c>
+      <c r="H37" s="8">
+        <v>40.049999999999997</v>
+      </c>
+      <c r="I37" s="8">
+        <v>1</v>
+      </c>
+      <c r="J37" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="K37" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L37" s="8">
+        <v>76</v>
+      </c>
+      <c r="M37" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N37" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A38" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="C38" s="8">
+        <v>1.6</v>
+      </c>
+      <c r="D38" s="8">
+        <v>2</v>
+      </c>
+      <c r="E38" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="F38" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="G38" s="8">
+        <v>15</v>
+      </c>
+      <c r="H38" s="8">
+        <v>7.9</v>
+      </c>
+      <c r="I38" s="8">
+        <v>-1</v>
+      </c>
+      <c r="J38" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K38" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L38" s="8">
+        <v>75</v>
+      </c>
+      <c r="M38" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N38" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A39" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="C39" s="8">
+        <v>0.4</v>
+      </c>
+      <c r="D39" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="E39" s="8">
+        <v>0</v>
+      </c>
+      <c r="F39" s="8">
+        <v>12.2</v>
+      </c>
+      <c r="G39" s="8">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="H39" s="8">
+        <v>0</v>
+      </c>
+      <c r="I39" s="8">
+        <v>-9</v>
+      </c>
+      <c r="J39" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K39" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L39" s="8">
+        <v>94</v>
+      </c>
+      <c r="M39" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N39" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A40" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="C40" s="8">
+        <v>0.3</v>
+      </c>
+      <c r="D40" s="8">
+        <v>1.8</v>
+      </c>
+      <c r="E40" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="F40" s="8">
+        <v>30</v>
+      </c>
+      <c r="G40" s="8">
+        <v>15</v>
+      </c>
+      <c r="H40" s="8">
+        <v>0</v>
+      </c>
+      <c r="I40" s="8">
+        <v>-8</v>
+      </c>
+      <c r="J40" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K40" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L40" s="8">
+        <v>97</v>
+      </c>
+      <c r="M40" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N40" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A41" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="C41" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="D41" s="8">
+        <v>5.4</v>
+      </c>
+      <c r="E41" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="F41" s="8">
+        <v>13</v>
+      </c>
+      <c r="G41" s="8">
+        <v>10</v>
+      </c>
+      <c r="H41" s="8">
+        <v>9</v>
+      </c>
+      <c r="I41" s="8">
+        <v>-4</v>
+      </c>
+      <c r="J41" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K41" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L41" s="8">
+        <v>87</v>
+      </c>
+      <c r="M41" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N41" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A42" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="C42" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D42" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="E42" s="8">
+        <v>0.02</v>
+      </c>
+      <c r="F42" s="8">
+        <v>13</v>
+      </c>
+      <c r="G42" s="8">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="H42" s="8">
+        <v>0</v>
+      </c>
+      <c r="I42" s="8">
+        <v>-6</v>
+      </c>
+      <c r="J42" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K42" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L42" s="8">
+        <v>82</v>
+      </c>
+      <c r="M42" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N42" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A43" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="C43" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="D43" s="8">
+        <v>10</v>
+      </c>
+      <c r="E43" s="8">
+        <v>0.02</v>
+      </c>
+      <c r="F43" s="8">
+        <v>11</v>
+      </c>
+      <c r="G43" s="8">
+        <v>8.5</v>
+      </c>
+      <c r="H43" s="8">
+        <v>20.5</v>
+      </c>
+      <c r="I43" s="8">
+        <v>1</v>
+      </c>
+      <c r="J43" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="K43" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L43" s="8">
+        <v>82</v>
+      </c>
+      <c r="M43" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N43" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A44" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="C44" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="D44" s="8">
+        <v>2.7</v>
+      </c>
+      <c r="E44" s="8">
+        <v>0.08</v>
+      </c>
+      <c r="F44" s="8">
+        <v>15.9</v>
+      </c>
+      <c r="G44" s="8">
+        <v>9.4</v>
+      </c>
+      <c r="H44" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="I44" s="8">
+        <v>-10</v>
+      </c>
+      <c r="J44" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K44" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L44" s="8">
+        <v>88</v>
+      </c>
+      <c r="M44" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N44" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A45" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="C45" s="8">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="D45" s="8">
+        <v>3.9</v>
+      </c>
+      <c r="E45" s="8">
+        <v>0.03</v>
+      </c>
+      <c r="F45" s="8">
+        <v>14</v>
+      </c>
+      <c r="G45" s="8">
+        <v>12</v>
+      </c>
+      <c r="H45" s="8">
+        <v>6</v>
+      </c>
+      <c r="I45" s="8">
+        <v>-1</v>
+      </c>
+      <c r="J45" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K45" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L45" s="8">
+        <v>82</v>
+      </c>
+      <c r="M45" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N45" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A46" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="C46" s="8">
+        <v>0.3</v>
+      </c>
+      <c r="D46" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="E46" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="F46" s="8">
+        <v>42</v>
+      </c>
+      <c r="G46" s="8">
+        <v>9.5</v>
+      </c>
+      <c r="H46" s="8">
+        <v>0</v>
+      </c>
+      <c r="I46" s="8">
+        <v>-3</v>
+      </c>
+      <c r="J46" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K46" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L46" s="8">
+        <v>97</v>
+      </c>
+      <c r="M46" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N46" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A47" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="C47" s="8">
+        <v>0.4</v>
+      </c>
+      <c r="D47" s="8">
+        <v>0</v>
+      </c>
+      <c r="E47" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="F47" s="8">
+        <v>20</v>
+      </c>
+      <c r="G47" s="8">
+        <v>11</v>
+      </c>
+      <c r="H47" s="8">
+        <v>0</v>
+      </c>
+      <c r="I47" s="8">
+        <v>-8</v>
+      </c>
+      <c r="J47" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K47" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L47" s="8">
+        <v>64</v>
+      </c>
+      <c r="M47" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N47" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A48" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="C48" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D48" s="8">
+        <v>2.7</v>
+      </c>
+      <c r="E48" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F48" s="8">
+        <v>5.7</v>
+      </c>
+      <c r="G48" s="8">
+        <v>11</v>
+      </c>
+      <c r="H48" s="8">
+        <v>0</v>
+      </c>
+      <c r="I48" s="8">
+        <v>0</v>
+      </c>
+      <c r="J48" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K48" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L48" s="8">
+        <v>97</v>
+      </c>
+      <c r="M48" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N48" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A49" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="C49" s="8">
+        <v>0.06</v>
+      </c>
+      <c r="D49" s="8">
+        <v>2.4</v>
+      </c>
+      <c r="E49" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="F49" s="8">
+        <v>18.600000000000001</v>
+      </c>
+      <c r="G49" s="8">
+        <v>15.5</v>
+      </c>
+      <c r="H49" s="8">
+        <v>0</v>
+      </c>
+      <c r="I49" s="8">
+        <v>-11</v>
+      </c>
+      <c r="J49" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K49" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L49" s="8">
+        <v>95</v>
+      </c>
+      <c r="M49" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N49" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A50" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="C50" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="D50" s="8">
+        <v>1.9</v>
+      </c>
+      <c r="E50" s="8">
+        <v>0.88</v>
+      </c>
+      <c r="F50" s="8">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="G50" s="8">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="H50" s="8">
+        <v>0</v>
+      </c>
+      <c r="I50" s="8">
+        <v>-1</v>
+      </c>
+      <c r="J50" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K50" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L50" s="8">
+        <v>93</v>
+      </c>
+      <c r="M50" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N50" s="8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A51" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="C51" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="D51" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="E51" s="8">
+        <v>0</v>
+      </c>
+      <c r="F51" s="8">
+        <v>13</v>
+      </c>
+      <c r="G51" s="8">
+        <v>8.9</v>
+      </c>
+      <c r="H51" s="8">
+        <v>0</v>
+      </c>
+      <c r="I51" s="8">
+        <v>-8</v>
+      </c>
+      <c r="J51" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K51" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="L51" s="8">
+        <v>99</v>
+      </c>
+      <c r="M51" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N51" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A52" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="C52" s="8">
+        <v>0.3</v>
+      </c>
+      <c r="D52" s="8">
+        <v>2.8</v>
+      </c>
+      <c r="E52" s="8">
+        <v>0.02</v>
+      </c>
+      <c r="F52" s="8">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="G52" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="H52" s="8">
+        <v>0</v>
+      </c>
+      <c r="I52" s="8">
+        <v>-1</v>
+      </c>
+      <c r="J52" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K52" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L52" s="8">
+        <v>97</v>
+      </c>
+      <c r="M52" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N52" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A53" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="C53" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="D53" s="8">
+        <v>2.7</v>
+      </c>
+      <c r="E53" s="8">
+        <v>0.71</v>
+      </c>
+      <c r="F53" s="8">
+        <v>12.8</v>
+      </c>
+      <c r="G53" s="8">
+        <v>18.7</v>
+      </c>
+      <c r="H53" s="8">
+        <v>0</v>
+      </c>
+      <c r="I53" s="8">
+        <v>-3</v>
+      </c>
+      <c r="J53" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K53" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L53" s="8">
+        <v>86</v>
+      </c>
+      <c r="M53" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N53" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A54" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="C54" s="8">
+        <v>1.21</v>
+      </c>
+      <c r="D54" s="8">
+        <v>0</v>
+      </c>
+      <c r="E54" s="8">
+        <v>0</v>
+      </c>
+      <c r="F54" s="8">
+        <v>16.3</v>
+      </c>
+      <c r="G54" s="8">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="H54" s="8">
+        <v>8</v>
+      </c>
+      <c r="I54" s="8">
+        <v>0</v>
+      </c>
+      <c r="J54" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K54" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L54" s="8">
+        <v>94</v>
+      </c>
+      <c r="M54" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N54" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A55" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="C55" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="D55" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="E55" s="8">
+        <v>0</v>
+      </c>
+      <c r="F55" s="8">
+        <v>14.4</v>
+      </c>
+      <c r="G55" s="8">
+        <v>5.6</v>
+      </c>
+      <c r="H55" s="8">
+        <v>20</v>
+      </c>
+      <c r="I55" s="8">
+        <v>-8</v>
+      </c>
+      <c r="J55" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K55" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="L55" s="8">
+        <v>86</v>
+      </c>
+      <c r="M55" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="N55" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A56" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="C56" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="D56" s="8">
+        <v>26</v>
+      </c>
+      <c r="E56" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F56" s="8">
+        <v>6.4</v>
+      </c>
+      <c r="G56" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="H56" s="8">
+        <v>11</v>
+      </c>
+      <c r="I56" s="8">
+        <v>20</v>
+      </c>
+      <c r="J56" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K56" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L56" s="8">
+        <v>45</v>
+      </c>
+      <c r="M56" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N56" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A57" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="C57" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D57" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="E57" s="8">
+        <v>0.43</v>
+      </c>
+      <c r="F57" s="8">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="G57" s="8">
+        <v>6.4</v>
+      </c>
+      <c r="H57" s="8">
+        <v>0</v>
+      </c>
+      <c r="I57" s="8">
+        <v>9</v>
+      </c>
+      <c r="J57" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K57" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L57" s="8">
+        <v>45</v>
+      </c>
+      <c r="M57" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N57" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A58" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="C58" s="8">
+        <v>0.3</v>
+      </c>
+      <c r="D58" s="8">
+        <v>22</v>
+      </c>
+      <c r="E58" s="8">
+        <v>0.74</v>
+      </c>
+      <c r="F58" s="8">
+        <v>6.4</v>
+      </c>
+      <c r="G58" s="8">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="H58" s="8">
+        <v>0</v>
+      </c>
+      <c r="I58" s="8">
+        <v>13</v>
+      </c>
+      <c r="J58" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="K58" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L58" s="8">
+        <v>45</v>
+      </c>
+      <c r="M58" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N58" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A59" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="B59" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C59" s="8">
+        <v>1.8</v>
+      </c>
+      <c r="D59" s="8">
+        <v>30</v>
+      </c>
+      <c r="E59" s="8">
+        <v>0</v>
+      </c>
+      <c r="F59" s="8">
+        <v>4.7</v>
+      </c>
+      <c r="G59" s="8">
+        <v>5.5</v>
+      </c>
+      <c r="H59" s="8">
+        <v>0</v>
+      </c>
+      <c r="I59" s="8">
+        <v>13</v>
+      </c>
+      <c r="J59" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="K59" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L59" s="8">
+        <v>45</v>
+      </c>
+      <c r="M59" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N59" s="8">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A60" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="C60" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="D60" s="8">
+        <v>25</v>
+      </c>
+      <c r="E60" s="8">
+        <v>0.88</v>
+      </c>
+      <c r="F60" s="8">
+        <v>9.4</v>
+      </c>
+      <c r="G60" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="H60" s="8">
+        <v>0</v>
+      </c>
+      <c r="I60" s="8">
+        <v>13</v>
+      </c>
+      <c r="J60" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="K60" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L60" s="8">
+        <v>45</v>
+      </c>
+      <c r="M60" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N60" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A61" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="C61" s="8">
+        <v>3.34</v>
+      </c>
+      <c r="D61" s="8">
+        <v>35.1</v>
+      </c>
+      <c r="E61" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="F61" s="8">
+        <v>8.1</v>
+      </c>
+      <c r="G61" s="8">
+        <v>3.6</v>
+      </c>
+      <c r="H61" s="8">
+        <v>16</v>
+      </c>
+      <c r="I61" s="8">
+        <v>20</v>
+      </c>
+      <c r="J61" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K61" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="L61" s="8">
+        <v>46</v>
+      </c>
+      <c r="M61" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N61" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A62" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="C62" s="8">
+        <v>10</v>
+      </c>
+      <c r="D62" s="8">
+        <v>25</v>
+      </c>
+      <c r="E62" s="8">
+        <v>0.73</v>
+      </c>
+      <c r="F62" s="8">
+        <v>7</v>
+      </c>
+      <c r="G62" s="8">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H62" s="8">
+        <v>0.4</v>
+      </c>
+      <c r="I62" s="8">
+        <v>24</v>
+      </c>
+      <c r="J62" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K62" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="L62" s="8">
+        <v>30</v>
+      </c>
+      <c r="M62" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N62" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A63" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="C63" s="8">
+        <v>10</v>
+      </c>
+      <c r="D63" s="8">
+        <v>25</v>
+      </c>
+      <c r="E63" s="8">
+        <v>0.68</v>
+      </c>
+      <c r="F63" s="8">
+        <v>7</v>
+      </c>
+      <c r="G63" s="8">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H63" s="8">
+        <v>0</v>
+      </c>
+      <c r="I63" s="8">
+        <v>23</v>
+      </c>
+      <c r="J63" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K63" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="L63" s="8">
+        <v>45</v>
+      </c>
+      <c r="M63" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N63" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C64" s="8">
+        <v>8.9</v>
+      </c>
+      <c r="D64" s="8">
+        <v>22</v>
+      </c>
+      <c r="E64" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="F64" s="8">
+        <v>7.4</v>
+      </c>
+      <c r="G64" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="H64" s="8">
+        <v>3.12</v>
+      </c>
+      <c r="I64" s="8">
+        <v>21</v>
+      </c>
+      <c r="J64" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K64" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="L64" s="8">
+        <v>45</v>
+      </c>
+      <c r="M64" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="N64" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A65" s="2"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
+      <c r="E65" s="2"/>
+      <c r="F65" s="2"/>
+      <c r="G65" s="2"/>
+      <c r="H65" s="2"/>
+      <c r="I65" s="2"/>
+      <c r="J65" s="2"/>
+      <c r="K65" s="2"/>
+      <c r="L65" s="2"/>
+      <c r="M65" s="2"/>
+      <c r="N65" s="2"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>